<commit_message>
Teachers: log in with the common code + own ΑΜ/ΑΦΜ; select/clear all; keep saved lists
- Clubs file, «Εκπαιδευτικοί»: optional «ΑΜ ή ΑΦΜ» column (digits, leading
  zeros dropped, one per teacher). Stored only as an HMAC; never sent back.
- Code login needs the teacher's ΑΜ/ΑΦΜ and shows only their own clubs;
  history names the teacher. Replaces the all-clubs common login.
- Teacher card: «Επιλογή όλων» (visible rows, if they fit), «Αποεπιλογή
  όλων», an unsaved-changes note, and the saved list is kept in the page
  (it was lost when switching clubs). Leaving or logging out with unsaved
  ticks asks first.
- Admin: ΑΜ/ΑΦΜ column in the teachers' table; template, help, docs, tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bv1rucCSvWvUULong8T8B
</commit_message>
<xml_diff>
--- a/platform/templates/omiloi_protypo.xlsx
+++ b/platform/templates/omiloi_protypo.xlsx
@@ -100,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,6 +115,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -619,7 +621,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>• Email: μόνο διευθύνσεις @sch.gr (με αυτό συνδέεται ο εκπαιδευτικός στην πλατφόρμα).</t>
+          <t>• Email: μόνο διευθύνσεις @sch.gr (για ειδοποιήσεις και τους προσωπικούς συνδέσμους εισόδου).</t>
         </is>
       </c>
     </row>
@@ -631,7 +633,11 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• ΑΜ ή ΑΦΜ: ο αριθμός μητρώου (μόνιμοι) ή το ΑΦΜ (αναπληρωτές) του εκπαιδευτικού. Μαζί με τον κοινό κωδικό εκπαιδευτικών, με αυτόν συνδέεται και βλέπει μόνο τους δικούς του ομίλους. Η πλατφόρμα δεν τον αποθηκεύει όπως είναι (μόνο κρυπτογραφικό αποτύπωμα).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -792,6 +798,11 @@
           <t>Όμιλος (έλεγχος)</t>
         </is>
       </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>ΑΜ ή ΑΦΜ</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -817,6 +828,11 @@
           <t>Θεατρική παράσταση</t>
         </is>
       </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>612345</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -840,6 +856,11 @@
       <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Θεατρική παράσταση</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>012345678</t>
         </is>
       </c>
     </row>
@@ -5465,7 +5486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E300"/>
+  <dimension ref="A1:F300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5473,6 +5494,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5501,6 +5523,11 @@
           <t>Όμιλος (έλεγχος)</t>
         </is>
       </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>ΑΜ ή ΑΦΜ</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="7" t="n"/>
@@ -5511,6 +5538,7 @@
         <f>IF(A2="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A2,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F2" s="11" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="n"/>
@@ -5521,6 +5549,7 @@
         <f>IF(A3="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A3,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="7" t="n"/>
@@ -5531,6 +5560,7 @@
         <f>IF(A4="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A4,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F4" s="11" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n"/>
@@ -5541,6 +5571,7 @@
         <f>IF(A5="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A5,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F5" s="11" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -5551,6 +5582,7 @@
         <f>IF(A6="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A6,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F6" s="11" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -5561,6 +5593,7 @@
         <f>IF(A7="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A7,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -5571,6 +5604,7 @@
         <f>IF(A8="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A8,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -5581,6 +5615,7 @@
         <f>IF(A9="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A9,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -5591,6 +5626,7 @@
         <f>IF(A10="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A10,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -5601,6 +5637,7 @@
         <f>IF(A11="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A11,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -5611,6 +5648,7 @@
         <f>IF(A12="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A12,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -5621,6 +5659,7 @@
         <f>IF(A13="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A13,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -5631,6 +5670,7 @@
         <f>IF(A14="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A14,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -5641,6 +5681,7 @@
         <f>IF(A15="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A15,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -5651,6 +5692,7 @@
         <f>IF(A16="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A16,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -5661,6 +5703,7 @@
         <f>IF(A17="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A17,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -5671,6 +5714,7 @@
         <f>IF(A18="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A18,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -5681,6 +5725,7 @@
         <f>IF(A19="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A19,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -5691,6 +5736,7 @@
         <f>IF(A20="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A20,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n"/>
@@ -5701,6 +5747,7 @@
         <f>IF(A21="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A21,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n"/>
@@ -5711,6 +5758,7 @@
         <f>IF(A22="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A22,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n"/>
@@ -5721,6 +5769,7 @@
         <f>IF(A23="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A23,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n"/>
@@ -5731,6 +5780,7 @@
         <f>IF(A24="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A24,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n"/>
@@ -5741,6 +5791,7 @@
         <f>IF(A25="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A25,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n"/>
@@ -5751,6 +5802,7 @@
         <f>IF(A26="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A26,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n"/>
@@ -5761,6 +5813,7 @@
         <f>IF(A27="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A27,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n"/>
@@ -5771,6 +5824,7 @@
         <f>IF(A28="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A28,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n"/>
@@ -5781,6 +5835,7 @@
         <f>IF(A29="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A29,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n"/>
@@ -5791,6 +5846,7 @@
         <f>IF(A30="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A30,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n"/>
@@ -5801,6 +5857,7 @@
         <f>IF(A31="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A31,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n"/>
@@ -5811,6 +5868,7 @@
         <f>IF(A32="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A32,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n"/>
@@ -5821,6 +5879,7 @@
         <f>IF(A33="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A33,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n"/>
@@ -5831,6 +5890,7 @@
         <f>IF(A34="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A34,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n"/>
@@ -5841,6 +5901,7 @@
         <f>IF(A35="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A35,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n"/>
@@ -5851,6 +5912,7 @@
         <f>IF(A36="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A36,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n"/>
@@ -5861,6 +5923,7 @@
         <f>IF(A37="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A37,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n"/>
@@ -5871,6 +5934,7 @@
         <f>IF(A38="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A38,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n"/>
@@ -5881,6 +5945,7 @@
         <f>IF(A39="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A39,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="n"/>
@@ -5891,6 +5956,7 @@
         <f>IF(A40="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A40,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="n"/>
@@ -5901,6 +5967,7 @@
         <f>IF(A41="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A41,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="n"/>
@@ -5911,6 +5978,7 @@
         <f>IF(A42="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A42,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="n"/>
@@ -5921,6 +5989,7 @@
         <f>IF(A43="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A43,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="n"/>
@@ -5931,6 +6000,7 @@
         <f>IF(A44="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A44,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="n"/>
@@ -5941,6 +6011,7 @@
         <f>IF(A45="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A45,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="n"/>
@@ -5951,6 +6022,7 @@
         <f>IF(A46="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A46,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="n"/>
@@ -5961,6 +6033,7 @@
         <f>IF(A47="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A47,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="n"/>
@@ -5971,6 +6044,7 @@
         <f>IF(A48="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A48,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="n"/>
@@ -5981,6 +6055,7 @@
         <f>IF(A49="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A49,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="n"/>
@@ -5991,6 +6066,7 @@
         <f>IF(A50="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A50,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="n"/>
@@ -6001,6 +6077,7 @@
         <f>IF(A51="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A51,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="n"/>
@@ -6011,6 +6088,7 @@
         <f>IF(A52="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A52,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="n"/>
@@ -6021,6 +6099,7 @@
         <f>IF(A53="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A53,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="n"/>
@@ -6031,6 +6110,7 @@
         <f>IF(A54="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A54,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="n"/>
@@ -6041,6 +6121,7 @@
         <f>IF(A55="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A55,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="n"/>
@@ -6051,6 +6132,7 @@
         <f>IF(A56="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A56,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="n"/>
@@ -6061,6 +6143,7 @@
         <f>IF(A57="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A57,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="n"/>
@@ -6071,6 +6154,7 @@
         <f>IF(A58="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A58,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="n"/>
@@ -6081,6 +6165,7 @@
         <f>IF(A59="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A59,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="n"/>
@@ -6091,6 +6176,7 @@
         <f>IF(A60="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A60,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="n"/>
@@ -6101,6 +6187,7 @@
         <f>IF(A61="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A61,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F61" s="11" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="n"/>
@@ -6111,6 +6198,7 @@
         <f>IF(A62="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A62,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F62" s="11" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="n"/>
@@ -6121,6 +6209,7 @@
         <f>IF(A63="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A63,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F63" s="11" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="n"/>
@@ -6131,6 +6220,7 @@
         <f>IF(A64="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A64,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F64" s="11" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="n"/>
@@ -6141,6 +6231,7 @@
         <f>IF(A65="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A65,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F65" s="11" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="n"/>
@@ -6151,6 +6242,7 @@
         <f>IF(A66="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A66,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F66" s="11" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="n"/>
@@ -6161,6 +6253,7 @@
         <f>IF(A67="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A67,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F67" s="11" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="n"/>
@@ -6171,6 +6264,7 @@
         <f>IF(A68="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A68,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F68" s="11" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="n"/>
@@ -6181,6 +6275,7 @@
         <f>IF(A69="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A69,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F69" s="11" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="n"/>
@@ -6191,6 +6286,7 @@
         <f>IF(A70="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A70,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F70" s="11" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="n"/>
@@ -6201,6 +6297,7 @@
         <f>IF(A71="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A71,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F71" s="11" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="n"/>
@@ -6211,6 +6308,7 @@
         <f>IF(A72="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A72,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F72" s="11" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="n"/>
@@ -6221,6 +6319,7 @@
         <f>IF(A73="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A73,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F73" s="11" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="n"/>
@@ -6231,6 +6330,7 @@
         <f>IF(A74="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A74,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F74" s="11" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="n"/>
@@ -6241,6 +6341,7 @@
         <f>IF(A75="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A75,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F75" s="11" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="n"/>
@@ -6251,6 +6352,7 @@
         <f>IF(A76="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A76,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F76" s="11" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="n"/>
@@ -6261,6 +6363,7 @@
         <f>IF(A77="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A77,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F77" s="11" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="n"/>
@@ -6271,6 +6374,7 @@
         <f>IF(A78="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A78,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F78" s="11" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="n"/>
@@ -6281,6 +6385,7 @@
         <f>IF(A79="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A79,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F79" s="11" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="n"/>
@@ -6291,6 +6396,7 @@
         <f>IF(A80="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A80,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F80" s="11" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="n"/>
@@ -6301,6 +6407,7 @@
         <f>IF(A81="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A81,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F81" s="11" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="n"/>
@@ -6311,6 +6418,7 @@
         <f>IF(A82="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A82,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F82" s="11" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="n"/>
@@ -6321,6 +6429,7 @@
         <f>IF(A83="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A83,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F83" s="11" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="n"/>
@@ -6331,6 +6440,7 @@
         <f>IF(A84="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A84,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F84" s="11" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="n"/>
@@ -6341,6 +6451,7 @@
         <f>IF(A85="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A85,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F85" s="11" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="n"/>
@@ -6351,6 +6462,7 @@
         <f>IF(A86="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A86,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F86" s="11" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="n"/>
@@ -6361,6 +6473,7 @@
         <f>IF(A87="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A87,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F87" s="11" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="n"/>
@@ -6371,6 +6484,7 @@
         <f>IF(A88="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A88,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F88" s="11" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="n"/>
@@ -6381,6 +6495,7 @@
         <f>IF(A89="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A89,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F89" s="11" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n"/>
@@ -6391,6 +6506,7 @@
         <f>IF(A90="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A90,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F90" s="11" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="n"/>
@@ -6401,6 +6517,7 @@
         <f>IF(A91="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A91,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F91" s="11" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="n"/>
@@ -6411,6 +6528,7 @@
         <f>IF(A92="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A92,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F92" s="11" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="n"/>
@@ -6421,6 +6539,7 @@
         <f>IF(A93="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A93,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F93" s="11" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="n"/>
@@ -6431,6 +6550,7 @@
         <f>IF(A94="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A94,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F94" s="11" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="n"/>
@@ -6441,6 +6561,7 @@
         <f>IF(A95="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A95,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F95" s="11" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="n"/>
@@ -6451,6 +6572,7 @@
         <f>IF(A96="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A96,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F96" s="11" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="n"/>
@@ -6461,6 +6583,7 @@
         <f>IF(A97="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A97,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F97" s="11" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="n"/>
@@ -6471,6 +6594,7 @@
         <f>IF(A98="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A98,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F98" s="11" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="n"/>
@@ -6481,6 +6605,7 @@
         <f>IF(A99="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A99,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F99" s="11" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="n"/>
@@ -6491,6 +6616,7 @@
         <f>IF(A100="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A100,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F100" s="11" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="n"/>
@@ -6501,6 +6627,7 @@
         <f>IF(A101="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A101,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F101" s="11" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="n"/>
@@ -6511,6 +6638,7 @@
         <f>IF(A102="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A102,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F102" s="11" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="n"/>
@@ -6521,6 +6649,7 @@
         <f>IF(A103="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A103,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F103" s="11" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="n"/>
@@ -6531,6 +6660,7 @@
         <f>IF(A104="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A104,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F104" s="11" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="n"/>
@@ -6541,6 +6671,7 @@
         <f>IF(A105="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A105,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F105" s="11" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="n"/>
@@ -6551,6 +6682,7 @@
         <f>IF(A106="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A106,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F106" s="11" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -6561,6 +6693,7 @@
         <f>IF(A107="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A107,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F107" s="11" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="n"/>
@@ -6571,6 +6704,7 @@
         <f>IF(A108="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A108,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F108" s="11" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="n"/>
@@ -6581,6 +6715,7 @@
         <f>IF(A109="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A109,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F109" s="11" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="n"/>
@@ -6591,6 +6726,7 @@
         <f>IF(A110="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A110,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F110" s="11" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="n"/>
@@ -6601,6 +6737,7 @@
         <f>IF(A111="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A111,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F111" s="11" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="n"/>
@@ -6611,6 +6748,7 @@
         <f>IF(A112="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A112,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F112" s="11" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="n"/>
@@ -6621,6 +6759,7 @@
         <f>IF(A113="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A113,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F113" s="11" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="n"/>
@@ -6631,6 +6770,7 @@
         <f>IF(A114="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A114,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F114" s="11" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="n"/>
@@ -6641,6 +6781,7 @@
         <f>IF(A115="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A115,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F115" s="11" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="n"/>
@@ -6651,6 +6792,7 @@
         <f>IF(A116="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A116,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F116" s="11" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="n"/>
@@ -6661,6 +6803,7 @@
         <f>IF(A117="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A117,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F117" s="11" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="n"/>
@@ -6671,6 +6814,7 @@
         <f>IF(A118="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A118,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F118" s="11" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="n"/>
@@ -6681,6 +6825,7 @@
         <f>IF(A119="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A119,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F119" s="11" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="n"/>
@@ -6691,6 +6836,7 @@
         <f>IF(A120="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A120,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F120" s="11" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="n"/>
@@ -6701,6 +6847,7 @@
         <f>IF(A121="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A121,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F121" s="11" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="n"/>
@@ -6711,6 +6858,7 @@
         <f>IF(A122="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A122,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F122" s="11" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n"/>
@@ -6721,6 +6869,7 @@
         <f>IF(A123="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A123,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F123" s="11" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="n"/>
@@ -6731,6 +6880,7 @@
         <f>IF(A124="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A124,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F124" s="11" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="n"/>
@@ -6741,6 +6891,7 @@
         <f>IF(A125="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A125,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F125" s="11" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="n"/>
@@ -6751,6 +6902,7 @@
         <f>IF(A126="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A126,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F126" s="11" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="n"/>
@@ -6761,6 +6913,7 @@
         <f>IF(A127="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A127,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F127" s="11" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="n"/>
@@ -6771,6 +6924,7 @@
         <f>IF(A128="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A128,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F128" s="11" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="n"/>
@@ -6781,6 +6935,7 @@
         <f>IF(A129="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A129,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F129" s="11" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="n"/>
@@ -6791,6 +6946,7 @@
         <f>IF(A130="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A130,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F130" s="11" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="n"/>
@@ -6801,6 +6957,7 @@
         <f>IF(A131="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A131,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F131" s="11" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="n"/>
@@ -6811,6 +6968,7 @@
         <f>IF(A132="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A132,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F132" s="11" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="n"/>
@@ -6821,6 +6979,7 @@
         <f>IF(A133="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A133,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F133" s="11" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="n"/>
@@ -6831,6 +6990,7 @@
         <f>IF(A134="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A134,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F134" s="11" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="n"/>
@@ -6841,6 +7001,7 @@
         <f>IF(A135="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A135,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F135" s="11" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="n"/>
@@ -6851,6 +7012,7 @@
         <f>IF(A136="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A136,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F136" s="11" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="n"/>
@@ -6861,6 +7023,7 @@
         <f>IF(A137="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A137,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F137" s="11" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="n"/>
@@ -6871,6 +7034,7 @@
         <f>IF(A138="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A138,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F138" s="11" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="n"/>
@@ -6881,6 +7045,7 @@
         <f>IF(A139="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A139,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F139" s="11" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="n"/>
@@ -6891,6 +7056,7 @@
         <f>IF(A140="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A140,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F140" s="11" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="n"/>
@@ -6901,6 +7067,7 @@
         <f>IF(A141="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A141,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F141" s="11" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="n"/>
@@ -6911,6 +7078,7 @@
         <f>IF(A142="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A142,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F142" s="11" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="n"/>
@@ -6921,6 +7089,7 @@
         <f>IF(A143="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A143,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F143" s="11" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="n"/>
@@ -6931,6 +7100,7 @@
         <f>IF(A144="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A144,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F144" s="11" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="n"/>
@@ -6941,6 +7111,7 @@
         <f>IF(A145="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A145,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F145" s="11" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="n"/>
@@ -6951,6 +7122,7 @@
         <f>IF(A146="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A146,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F146" s="11" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="n"/>
@@ -6961,6 +7133,7 @@
         <f>IF(A147="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A147,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F147" s="11" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="n"/>
@@ -6971,6 +7144,7 @@
         <f>IF(A148="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A148,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F148" s="11" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="n"/>
@@ -6981,6 +7155,7 @@
         <f>IF(A149="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A149,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F149" s="11" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="n"/>
@@ -6991,6 +7166,7 @@
         <f>IF(A150="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A150,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F150" s="11" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="n"/>
@@ -7001,6 +7177,7 @@
         <f>IF(A151="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A151,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F151" s="11" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="n"/>
@@ -7011,6 +7188,7 @@
         <f>IF(A152="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A152,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F152" s="11" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="n"/>
@@ -7021,6 +7199,7 @@
         <f>IF(A153="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A153,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F153" s="11" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="n"/>
@@ -7031,6 +7210,7 @@
         <f>IF(A154="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A154,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F154" s="11" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="n"/>
@@ -7041,6 +7221,7 @@
         <f>IF(A155="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A155,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F155" s="11" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="n"/>
@@ -7051,6 +7232,7 @@
         <f>IF(A156="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A156,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F156" s="11" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="n"/>
@@ -7061,6 +7243,7 @@
         <f>IF(A157="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A157,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F157" s="11" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="n"/>
@@ -7071,6 +7254,7 @@
         <f>IF(A158="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A158,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F158" s="11" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="n"/>
@@ -7081,6 +7265,7 @@
         <f>IF(A159="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A159,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F159" s="11" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="n"/>
@@ -7091,6 +7276,7 @@
         <f>IF(A160="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A160,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F160" s="11" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="n"/>
@@ -7101,6 +7287,7 @@
         <f>IF(A161="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A161,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F161" s="11" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="n"/>
@@ -7111,6 +7298,7 @@
         <f>IF(A162="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A162,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F162" s="11" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="n"/>
@@ -7121,6 +7309,7 @@
         <f>IF(A163="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A163,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F163" s="11" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="n"/>
@@ -7131,6 +7320,7 @@
         <f>IF(A164="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A164,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F164" s="11" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="n"/>
@@ -7141,6 +7331,7 @@
         <f>IF(A165="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A165,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F165" s="11" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="n"/>
@@ -7151,6 +7342,7 @@
         <f>IF(A166="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A166,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F166" s="11" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="n"/>
@@ -7161,6 +7353,7 @@
         <f>IF(A167="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A167,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F167" s="11" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="n"/>
@@ -7171,6 +7364,7 @@
         <f>IF(A168="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A168,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F168" s="11" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="n"/>
@@ -7181,6 +7375,7 @@
         <f>IF(A169="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A169,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F169" s="11" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="n"/>
@@ -7191,6 +7386,7 @@
         <f>IF(A170="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A170,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F170" s="11" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="n"/>
@@ -7201,6 +7397,7 @@
         <f>IF(A171="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A171,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F171" s="11" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="n"/>
@@ -7211,6 +7408,7 @@
         <f>IF(A172="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A172,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F172" s="11" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="n"/>
@@ -7221,6 +7419,7 @@
         <f>IF(A173="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A173,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F173" s="11" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="n"/>
@@ -7231,6 +7430,7 @@
         <f>IF(A174="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A174,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F174" s="11" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="n"/>
@@ -7241,6 +7441,7 @@
         <f>IF(A175="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A175,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F175" s="11" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="n"/>
@@ -7251,6 +7452,7 @@
         <f>IF(A176="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A176,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F176" s="11" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="n"/>
@@ -7261,6 +7463,7 @@
         <f>IF(A177="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A177,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F177" s="11" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="n"/>
@@ -7271,6 +7474,7 @@
         <f>IF(A178="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A178,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F178" s="11" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="n"/>
@@ -7281,6 +7485,7 @@
         <f>IF(A179="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A179,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F179" s="11" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="n"/>
@@ -7291,6 +7496,7 @@
         <f>IF(A180="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A180,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F180" s="11" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="n"/>
@@ -7301,6 +7507,7 @@
         <f>IF(A181="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A181,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F181" s="11" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="n"/>
@@ -7311,6 +7518,7 @@
         <f>IF(A182="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A182,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F182" s="11" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="n"/>
@@ -7321,6 +7529,7 @@
         <f>IF(A183="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A183,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F183" s="11" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="n"/>
@@ -7331,6 +7540,7 @@
         <f>IF(A184="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A184,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F184" s="11" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="n"/>
@@ -7341,6 +7551,7 @@
         <f>IF(A185="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A185,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F185" s="11" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="n"/>
@@ -7351,6 +7562,7 @@
         <f>IF(A186="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A186,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F186" s="11" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="n"/>
@@ -7361,6 +7573,7 @@
         <f>IF(A187="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A187,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F187" s="11" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="n"/>
@@ -7371,6 +7584,7 @@
         <f>IF(A188="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A188,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F188" s="11" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="n"/>
@@ -7381,6 +7595,7 @@
         <f>IF(A189="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A189,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F189" s="11" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="n"/>
@@ -7391,6 +7606,7 @@
         <f>IF(A190="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A190,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F190" s="11" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="n"/>
@@ -7401,6 +7617,7 @@
         <f>IF(A191="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A191,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F191" s="11" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="n"/>
@@ -7411,6 +7628,7 @@
         <f>IF(A192="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A192,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F192" s="11" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="n"/>
@@ -7421,6 +7639,7 @@
         <f>IF(A193="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A193,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F193" s="11" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="n"/>
@@ -7431,6 +7650,7 @@
         <f>IF(A194="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A194,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F194" s="11" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="n"/>
@@ -7441,6 +7661,7 @@
         <f>IF(A195="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A195,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F195" s="11" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="n"/>
@@ -7451,6 +7672,7 @@
         <f>IF(A196="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A196,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F196" s="11" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="n"/>
@@ -7461,6 +7683,7 @@
         <f>IF(A197="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A197,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F197" s="11" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="n"/>
@@ -7471,6 +7694,7 @@
         <f>IF(A198="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A198,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F198" s="11" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="n"/>
@@ -7481,6 +7705,7 @@
         <f>IF(A199="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A199,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F199" s="11" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="n"/>
@@ -7491,6 +7716,7 @@
         <f>IF(A200="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A200,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F200" s="11" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="n"/>
@@ -7501,6 +7727,7 @@
         <f>IF(A201="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A201,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F201" s="11" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="n"/>
@@ -7511,6 +7738,7 @@
         <f>IF(A202="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A202,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F202" s="11" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="n"/>
@@ -7521,6 +7749,7 @@
         <f>IF(A203="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A203,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F203" s="11" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="n"/>
@@ -7531,6 +7760,7 @@
         <f>IF(A204="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A204,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F204" s="11" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="n"/>
@@ -7541,6 +7771,7 @@
         <f>IF(A205="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A205,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F205" s="11" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="n"/>
@@ -7551,6 +7782,7 @@
         <f>IF(A206="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A206,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F206" s="11" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="n"/>
@@ -7561,6 +7793,7 @@
         <f>IF(A207="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A207,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F207" s="11" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="n"/>
@@ -7571,6 +7804,7 @@
         <f>IF(A208="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A208,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F208" s="11" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="n"/>
@@ -7581,6 +7815,7 @@
         <f>IF(A209="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A209,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F209" s="11" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="n"/>
@@ -7591,6 +7826,7 @@
         <f>IF(A210="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A210,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F210" s="11" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="7" t="n"/>
@@ -7601,6 +7837,7 @@
         <f>IF(A211="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A211,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F211" s="11" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="n"/>
@@ -7611,6 +7848,7 @@
         <f>IF(A212="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A212,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F212" s="11" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="n"/>
@@ -7621,6 +7859,7 @@
         <f>IF(A213="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A213,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F213" s="11" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="7" t="n"/>
@@ -7631,6 +7870,7 @@
         <f>IF(A214="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A214,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F214" s="11" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="n"/>
@@ -7641,6 +7881,7 @@
         <f>IF(A215="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A215,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F215" s="11" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="7" t="n"/>
@@ -7651,6 +7892,7 @@
         <f>IF(A216="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A216,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F216" s="11" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="7" t="n"/>
@@ -7661,6 +7903,7 @@
         <f>IF(A217="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A217,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F217" s="11" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="7" t="n"/>
@@ -7671,6 +7914,7 @@
         <f>IF(A218="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A218,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F218" s="11" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="7" t="n"/>
@@ -7681,6 +7925,7 @@
         <f>IF(A219="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A219,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F219" s="11" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="7" t="n"/>
@@ -7691,6 +7936,7 @@
         <f>IF(A220="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A220,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F220" s="11" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="7" t="n"/>
@@ -7701,6 +7947,7 @@
         <f>IF(A221="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A221,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F221" s="11" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="n"/>
@@ -7711,6 +7958,7 @@
         <f>IF(A222="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A222,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F222" s="11" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="7" t="n"/>
@@ -7721,6 +7969,7 @@
         <f>IF(A223="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A223,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F223" s="11" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="7" t="n"/>
@@ -7731,6 +7980,7 @@
         <f>IF(A224="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A224,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F224" s="11" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="7" t="n"/>
@@ -7741,6 +7991,7 @@
         <f>IF(A225="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A225,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F225" s="11" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="7" t="n"/>
@@ -7751,6 +8002,7 @@
         <f>IF(A226="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A226,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F226" s="11" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="7" t="n"/>
@@ -7761,6 +8013,7 @@
         <f>IF(A227="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A227,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F227" s="11" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="7" t="n"/>
@@ -7771,6 +8024,7 @@
         <f>IF(A228="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A228,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F228" s="11" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="7" t="n"/>
@@ -7781,6 +8035,7 @@
         <f>IF(A229="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A229,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F229" s="11" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="7" t="n"/>
@@ -7791,6 +8046,7 @@
         <f>IF(A230="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A230,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F230" s="11" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="7" t="n"/>
@@ -7801,6 +8057,7 @@
         <f>IF(A231="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A231,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F231" s="11" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="7" t="n"/>
@@ -7811,6 +8068,7 @@
         <f>IF(A232="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A232,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F232" s="11" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="7" t="n"/>
@@ -7821,6 +8079,7 @@
         <f>IF(A233="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A233,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F233" s="11" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="7" t="n"/>
@@ -7831,6 +8090,7 @@
         <f>IF(A234="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A234,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F234" s="11" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="7" t="n"/>
@@ -7841,6 +8101,7 @@
         <f>IF(A235="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A235,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F235" s="11" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="7" t="n"/>
@@ -7851,6 +8112,7 @@
         <f>IF(A236="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A236,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F236" s="11" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="7" t="n"/>
@@ -7861,6 +8123,7 @@
         <f>IF(A237="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A237,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F237" s="11" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="7" t="n"/>
@@ -7871,6 +8134,7 @@
         <f>IF(A238="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A238,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F238" s="11" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="7" t="n"/>
@@ -7881,6 +8145,7 @@
         <f>IF(A239="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A239,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F239" s="11" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="7" t="n"/>
@@ -7891,6 +8156,7 @@
         <f>IF(A240="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A240,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F240" s="11" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="7" t="n"/>
@@ -7901,6 +8167,7 @@
         <f>IF(A241="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A241,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F241" s="11" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="7" t="n"/>
@@ -7911,6 +8178,7 @@
         <f>IF(A242="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A242,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F242" s="11" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="7" t="n"/>
@@ -7921,6 +8189,7 @@
         <f>IF(A243="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A243,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F243" s="11" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="7" t="n"/>
@@ -7931,6 +8200,7 @@
         <f>IF(A244="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A244,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F244" s="11" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="7" t="n"/>
@@ -7941,6 +8211,7 @@
         <f>IF(A245="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A245,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F245" s="11" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="7" t="n"/>
@@ -7951,6 +8222,7 @@
         <f>IF(A246="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A246,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F246" s="11" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="7" t="n"/>
@@ -7961,6 +8233,7 @@
         <f>IF(A247="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A247,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F247" s="11" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="7" t="n"/>
@@ -7971,6 +8244,7 @@
         <f>IF(A248="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A248,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F248" s="11" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="7" t="n"/>
@@ -7981,6 +8255,7 @@
         <f>IF(A249="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A249,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F249" s="11" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="7" t="n"/>
@@ -7991,6 +8266,7 @@
         <f>IF(A250="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A250,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F250" s="11" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="7" t="n"/>
@@ -8001,6 +8277,7 @@
         <f>IF(A251="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A251,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F251" s="11" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="7" t="n"/>
@@ -8011,6 +8288,7 @@
         <f>IF(A252="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A252,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F252" s="11" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="7" t="n"/>
@@ -8021,6 +8299,7 @@
         <f>IF(A253="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A253,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F253" s="11" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="7" t="n"/>
@@ -8031,6 +8310,7 @@
         <f>IF(A254="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A254,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F254" s="11" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="7" t="n"/>
@@ -8041,6 +8321,7 @@
         <f>IF(A255="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A255,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F255" s="11" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="7" t="n"/>
@@ -8051,6 +8332,7 @@
         <f>IF(A256="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A256,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F256" s="11" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="7" t="n"/>
@@ -8061,6 +8343,7 @@
         <f>IF(A257="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A257,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F257" s="11" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="7" t="n"/>
@@ -8071,6 +8354,7 @@
         <f>IF(A258="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A258,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F258" s="11" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="7" t="n"/>
@@ -8081,6 +8365,7 @@
         <f>IF(A259="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A259,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F259" s="11" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="7" t="n"/>
@@ -8091,6 +8376,7 @@
         <f>IF(A260="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A260,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F260" s="11" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="7" t="n"/>
@@ -8101,6 +8387,7 @@
         <f>IF(A261="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A261,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F261" s="11" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="7" t="n"/>
@@ -8111,6 +8398,7 @@
         <f>IF(A262="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A262,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F262" s="11" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="7" t="n"/>
@@ -8121,6 +8409,7 @@
         <f>IF(A263="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A263,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F263" s="11" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="7" t="n"/>
@@ -8131,6 +8420,7 @@
         <f>IF(A264="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A264,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F264" s="11" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="7" t="n"/>
@@ -8141,6 +8431,7 @@
         <f>IF(A265="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A265,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F265" s="11" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="7" t="n"/>
@@ -8151,6 +8442,7 @@
         <f>IF(A266="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A266,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F266" s="11" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="7" t="n"/>
@@ -8161,6 +8453,7 @@
         <f>IF(A267="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A267,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F267" s="11" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="7" t="n"/>
@@ -8171,6 +8464,7 @@
         <f>IF(A268="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A268,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F268" s="11" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="7" t="n"/>
@@ -8181,6 +8475,7 @@
         <f>IF(A269="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A269,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F269" s="11" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="7" t="n"/>
@@ -8191,6 +8486,7 @@
         <f>IF(A270="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A270,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F270" s="11" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="7" t="n"/>
@@ -8201,6 +8497,7 @@
         <f>IF(A271="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A271,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F271" s="11" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="7" t="n"/>
@@ -8211,6 +8508,7 @@
         <f>IF(A272="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A272,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F272" s="11" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="7" t="n"/>
@@ -8221,6 +8519,7 @@
         <f>IF(A273="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A273,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F273" s="11" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="7" t="n"/>
@@ -8231,6 +8530,7 @@
         <f>IF(A274="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A274,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F274" s="11" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="7" t="n"/>
@@ -8241,6 +8541,7 @@
         <f>IF(A275="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A275,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F275" s="11" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="7" t="n"/>
@@ -8251,6 +8552,7 @@
         <f>IF(A276="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A276,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F276" s="11" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="7" t="n"/>
@@ -8261,6 +8563,7 @@
         <f>IF(A277="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A277,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F277" s="11" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="7" t="n"/>
@@ -8271,6 +8574,7 @@
         <f>IF(A278="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A278,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F278" s="11" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="7" t="n"/>
@@ -8281,6 +8585,7 @@
         <f>IF(A279="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A279,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F279" s="11" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="7" t="n"/>
@@ -8291,6 +8596,7 @@
         <f>IF(A280="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A280,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F280" s="11" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="7" t="n"/>
@@ -8301,6 +8607,7 @@
         <f>IF(A281="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A281,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F281" s="11" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="7" t="n"/>
@@ -8311,6 +8618,7 @@
         <f>IF(A282="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A282,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F282" s="11" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="7" t="n"/>
@@ -8321,6 +8629,7 @@
         <f>IF(A283="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A283,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F283" s="11" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="7" t="n"/>
@@ -8331,6 +8640,7 @@
         <f>IF(A284="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A284,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F284" s="11" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="7" t="n"/>
@@ -8341,6 +8651,7 @@
         <f>IF(A285="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A285,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F285" s="11" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="7" t="n"/>
@@ -8351,6 +8662,7 @@
         <f>IF(A286="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A286,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F286" s="11" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="7" t="n"/>
@@ -8361,6 +8673,7 @@
         <f>IF(A287="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A287,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F287" s="11" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="7" t="n"/>
@@ -8371,6 +8684,7 @@
         <f>IF(A288="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A288,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F288" s="11" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="7" t="n"/>
@@ -8381,6 +8695,7 @@
         <f>IF(A289="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A289,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F289" s="11" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="7" t="n"/>
@@ -8391,6 +8706,7 @@
         <f>IF(A290="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A290,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F290" s="11" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="7" t="n"/>
@@ -8401,6 +8717,7 @@
         <f>IF(A291="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A291,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F291" s="11" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="7" t="n"/>
@@ -8411,6 +8728,7 @@
         <f>IF(A292="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A292,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F292" s="11" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="7" t="n"/>
@@ -8421,6 +8739,7 @@
         <f>IF(A293="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A293,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F293" s="11" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="7" t="n"/>
@@ -8431,6 +8750,7 @@
         <f>IF(A294="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A294,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F294" s="11" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="7" t="n"/>
@@ -8441,6 +8761,7 @@
         <f>IF(A295="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A295,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F295" s="11" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="7" t="n"/>
@@ -8451,6 +8772,7 @@
         <f>IF(A296="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A296,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F296" s="11" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="7" t="n"/>
@@ -8461,6 +8783,7 @@
         <f>IF(A297="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A297,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F297" s="11" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="7" t="n"/>
@@ -8471,6 +8794,7 @@
         <f>IF(A298="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A298,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F298" s="11" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="7" t="n"/>
@@ -8481,6 +8805,7 @@
         <f>IF(A299="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A299,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F299" s="11" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="7" t="n"/>
@@ -8491,6 +8816,7 @@
         <f>IF(A300="","",IFERROR(INDEX('Όμιλοι'!$B$2:$B$300,MATCH(A300,'Όμιλοι'!$A$2:$A$300,0)),";;"))</f>
         <v/>
       </c>
+      <c r="F300" s="11" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E300">

</xml_diff>